<commit_message>
GOT FL1 COMP BOXPLOT!!!
</commit_message>
<xml_diff>
--- a/data/FirebreakData_Nov2026.xlsx
+++ b/data/FirebreakData_Nov2026.xlsx
@@ -5152,18 +5152,26 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="3"/>
+      <c r="A80" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="B80" s="3"/>
       <c r="C80" s="3"/>
       <c r="D80" s="3"/>
-      <c r="E80" s="3"/>
-      <c r="F80" s="3"/>
+      <c r="E80" s="2">
+        <v>1.0</v>
+      </c>
+      <c r="F80" s="2"/>
       <c r="G80" s="3"/>
       <c r="H80" s="3"/>
-      <c r="I80" s="3"/>
-      <c r="J80" s="3"/>
-      <c r="K80" s="3"/>
-      <c r="L80" s="3"/>
+      <c r="I80" s="2">
+        <v>1.0</v>
+      </c>
+      <c r="J80" s="2"/>
+      <c r="K80" s="2">
+        <v>1.0</v>
+      </c>
+      <c r="L80" s="2"/>
       <c r="M80" s="3"/>
       <c r="N80" s="3"/>
       <c r="O80" s="3"/>
@@ -5173,6 +5181,7 @@
       <c r="S80" s="3"/>
       <c r="T80" s="3"/>
       <c r="U80" s="3"/>
+      <c r="V80" s="3"/>
     </row>
     <row r="81">
       <c r="A81" s="3"/>
@@ -5341,38 +5350,6 @@
       <c r="U85" s="3"/>
       <c r="V85" s="3"/>
     </row>
-    <row r="86">
-      <c r="A86" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B86" s="3"/>
-      <c r="C86" s="3"/>
-      <c r="D86" s="3"/>
-      <c r="E86" s="2">
-        <v>1.0</v>
-      </c>
-      <c r="F86" s="2"/>
-      <c r="G86" s="3"/>
-      <c r="H86" s="3"/>
-      <c r="I86" s="2">
-        <v>1.0</v>
-      </c>
-      <c r="J86" s="2"/>
-      <c r="K86" s="2">
-        <v>1.0</v>
-      </c>
-      <c r="L86" s="2"/>
-      <c r="M86" s="3"/>
-      <c r="N86" s="3"/>
-      <c r="O86" s="3"/>
-      <c r="P86" s="3"/>
-      <c r="Q86" s="3"/>
-      <c r="R86" s="3"/>
-      <c r="S86" s="3"/>
-      <c r="T86" s="3"/>
-      <c r="U86" s="3"/>
-      <c r="V86" s="3"/>
-    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -7490,7 +7467,9 @@
       <c r="U78" s="3"/>
     </row>
     <row r="79">
-      <c r="A79" s="3"/>
+      <c r="A79" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="B79" s="3"/>
       <c r="C79" s="3"/>
       <c r="D79" s="3"/>
@@ -7511,6 +7490,7 @@
       <c r="S79" s="3"/>
       <c r="T79" s="3"/>
       <c r="U79" s="3"/>
+      <c r="V79" s="3"/>
     </row>
     <row r="80">
       <c r="A80" s="3"/>
@@ -7720,32 +7700,6 @@
       </c>
       <c r="V85" s="2"/>
     </row>
-    <row r="86">
-      <c r="A86" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B86" s="3"/>
-      <c r="C86" s="3"/>
-      <c r="D86" s="3"/>
-      <c r="E86" s="3"/>
-      <c r="F86" s="3"/>
-      <c r="G86" s="3"/>
-      <c r="H86" s="3"/>
-      <c r="I86" s="3"/>
-      <c r="J86" s="3"/>
-      <c r="K86" s="3"/>
-      <c r="L86" s="3"/>
-      <c r="M86" s="3"/>
-      <c r="N86" s="3"/>
-      <c r="O86" s="3"/>
-      <c r="P86" s="3"/>
-      <c r="Q86" s="3"/>
-      <c r="R86" s="3"/>
-      <c r="S86" s="3"/>
-      <c r="T86" s="3"/>
-      <c r="U86" s="3"/>
-      <c r="V86" s="3"/>
-    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -9845,7 +9799,9 @@
       <c r="U78" s="3"/>
     </row>
     <row r="79">
-      <c r="A79" s="3"/>
+      <c r="A79" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="B79" s="3"/>
       <c r="C79" s="3"/>
       <c r="D79" s="3"/>
@@ -9866,6 +9822,7 @@
       <c r="S79" s="3"/>
       <c r="T79" s="3"/>
       <c r="U79" s="3"/>
+      <c r="V79" s="3"/>
     </row>
     <row r="80">
       <c r="A80" s="3"/>
@@ -10069,32 +10026,6 @@
       </c>
       <c r="V85" s="2"/>
     </row>
-    <row r="86">
-      <c r="A86" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B86" s="3"/>
-      <c r="C86" s="3"/>
-      <c r="D86" s="3"/>
-      <c r="E86" s="3"/>
-      <c r="F86" s="3"/>
-      <c r="G86" s="3"/>
-      <c r="H86" s="3"/>
-      <c r="I86" s="3"/>
-      <c r="J86" s="3"/>
-      <c r="K86" s="3"/>
-      <c r="L86" s="3"/>
-      <c r="M86" s="3"/>
-      <c r="N86" s="3"/>
-      <c r="O86" s="3"/>
-      <c r="P86" s="3"/>
-      <c r="Q86" s="3"/>
-      <c r="R86" s="3"/>
-      <c r="S86" s="3"/>
-      <c r="T86" s="3"/>
-      <c r="U86" s="3"/>
-      <c r="V86" s="3"/>
-    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -12220,7 +12151,9 @@
       <c r="U78" s="3"/>
     </row>
     <row r="79">
-      <c r="A79" s="3"/>
+      <c r="A79" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="B79" s="3"/>
       <c r="C79" s="3"/>
       <c r="D79" s="3"/>
@@ -12241,6 +12174,7 @@
       <c r="S79" s="3"/>
       <c r="T79" s="3"/>
       <c r="U79" s="3"/>
+      <c r="V79" s="3"/>
     </row>
     <row r="80">
       <c r="A80" s="3"/>
@@ -12452,32 +12386,6 @@
       </c>
       <c r="V85" s="2"/>
     </row>
-    <row r="86">
-      <c r="A86" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B86" s="3"/>
-      <c r="C86" s="3"/>
-      <c r="D86" s="3"/>
-      <c r="E86" s="3"/>
-      <c r="F86" s="3"/>
-      <c r="G86" s="3"/>
-      <c r="H86" s="3"/>
-      <c r="I86" s="3"/>
-      <c r="J86" s="3"/>
-      <c r="K86" s="3"/>
-      <c r="L86" s="3"/>
-      <c r="M86" s="3"/>
-      <c r="N86" s="3"/>
-      <c r="O86" s="3"/>
-      <c r="P86" s="3"/>
-      <c r="Q86" s="3"/>
-      <c r="R86" s="3"/>
-      <c r="S86" s="3"/>
-      <c r="T86" s="3"/>
-      <c r="U86" s="3"/>
-      <c r="V86" s="3"/>
-    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -14597,7 +14505,9 @@
       <c r="U78" s="3"/>
     </row>
     <row r="79">
-      <c r="A79" s="3"/>
+      <c r="A79" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="B79" s="3"/>
       <c r="C79" s="3"/>
       <c r="D79" s="3"/>
@@ -14618,6 +14528,7 @@
       <c r="S79" s="3"/>
       <c r="T79" s="3"/>
       <c r="U79" s="3"/>
+      <c r="V79" s="3"/>
     </row>
     <row r="80">
       <c r="A80" s="3"/>
@@ -14801,32 +14712,6 @@
       <c r="U85" s="3"/>
       <c r="V85" s="3"/>
     </row>
-    <row r="86">
-      <c r="A86" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B86" s="3"/>
-      <c r="C86" s="3"/>
-      <c r="D86" s="3"/>
-      <c r="E86" s="3"/>
-      <c r="F86" s="3"/>
-      <c r="G86" s="3"/>
-      <c r="H86" s="3"/>
-      <c r="I86" s="3"/>
-      <c r="J86" s="3"/>
-      <c r="K86" s="3"/>
-      <c r="L86" s="3"/>
-      <c r="M86" s="3"/>
-      <c r="N86" s="3"/>
-      <c r="O86" s="3"/>
-      <c r="P86" s="3"/>
-      <c r="Q86" s="3"/>
-      <c r="R86" s="3"/>
-      <c r="S86" s="3"/>
-      <c r="T86" s="3"/>
-      <c r="U86" s="3"/>
-      <c r="V86" s="3"/>
-    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -16951,7 +16836,9 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="3"/>
+      <c r="A80" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="B80" s="3"/>
       <c r="C80" s="3"/>
       <c r="D80" s="3"/>
@@ -16972,6 +16859,7 @@
       <c r="S80" s="3"/>
       <c r="T80" s="3"/>
       <c r="U80" s="3"/>
+      <c r="V80" s="3"/>
     </row>
     <row r="81">
       <c r="A81" s="3"/>
@@ -17142,32 +17030,6 @@
       <c r="U85" s="3"/>
       <c r="V85" s="3"/>
     </row>
-    <row r="86">
-      <c r="A86" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B86" s="3"/>
-      <c r="C86" s="3"/>
-      <c r="D86" s="3"/>
-      <c r="E86" s="3"/>
-      <c r="F86" s="3"/>
-      <c r="G86" s="3"/>
-      <c r="H86" s="3"/>
-      <c r="I86" s="3"/>
-      <c r="J86" s="3"/>
-      <c r="K86" s="3"/>
-      <c r="L86" s="3"/>
-      <c r="M86" s="3"/>
-      <c r="N86" s="3"/>
-      <c r="O86" s="3"/>
-      <c r="P86" s="3"/>
-      <c r="Q86" s="3"/>
-      <c r="R86" s="3"/>
-      <c r="S86" s="3"/>
-      <c r="T86" s="3"/>
-      <c r="U86" s="3"/>
-      <c r="V86" s="3"/>
-    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -19249,7 +19111,9 @@
       <c r="U78" s="3"/>
     </row>
     <row r="79">
-      <c r="A79" s="3"/>
+      <c r="A79" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="B79" s="3"/>
       <c r="C79" s="3"/>
       <c r="D79" s="3"/>
@@ -19270,6 +19134,7 @@
       <c r="S79" s="3"/>
       <c r="T79" s="3"/>
       <c r="U79" s="3"/>
+      <c r="V79" s="3"/>
     </row>
     <row r="80">
       <c r="A80" s="3"/>
@@ -19461,32 +19326,6 @@
       <c r="U85" s="3"/>
       <c r="V85" s="3"/>
     </row>
-    <row r="86">
-      <c r="A86" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B86" s="3"/>
-      <c r="C86" s="3"/>
-      <c r="D86" s="3"/>
-      <c r="E86" s="3"/>
-      <c r="F86" s="3"/>
-      <c r="G86" s="3"/>
-      <c r="H86" s="3"/>
-      <c r="I86" s="3"/>
-      <c r="J86" s="3"/>
-      <c r="K86" s="3"/>
-      <c r="L86" s="3"/>
-      <c r="M86" s="3"/>
-      <c r="N86" s="3"/>
-      <c r="O86" s="3"/>
-      <c r="P86" s="3"/>
-      <c r="Q86" s="3"/>
-      <c r="R86" s="3"/>
-      <c r="S86" s="3"/>
-      <c r="T86" s="3"/>
-      <c r="U86" s="3"/>
-      <c r="V86" s="3"/>
-    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -21596,7 +21435,9 @@
       <c r="U78" s="3"/>
     </row>
     <row r="79">
-      <c r="A79" s="3"/>
+      <c r="A79" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="B79" s="3"/>
       <c r="C79" s="3"/>
       <c r="D79" s="3"/>
@@ -21617,6 +21458,7 @@
       <c r="S79" s="3"/>
       <c r="T79" s="3"/>
       <c r="U79" s="3"/>
+      <c r="V79" s="3"/>
     </row>
     <row r="80">
       <c r="A80" s="3"/>
@@ -21808,32 +21650,6 @@
       <c r="U85" s="3"/>
       <c r="V85" s="3"/>
     </row>
-    <row r="86">
-      <c r="A86" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B86" s="3"/>
-      <c r="C86" s="3"/>
-      <c r="D86" s="3"/>
-      <c r="E86" s="3"/>
-      <c r="F86" s="3"/>
-      <c r="G86" s="3"/>
-      <c r="H86" s="3"/>
-      <c r="I86" s="3"/>
-      <c r="J86" s="3"/>
-      <c r="K86" s="3"/>
-      <c r="L86" s="3"/>
-      <c r="M86" s="3"/>
-      <c r="N86" s="3"/>
-      <c r="O86" s="3"/>
-      <c r="P86" s="3"/>
-      <c r="Q86" s="3"/>
-      <c r="R86" s="3"/>
-      <c r="S86" s="3"/>
-      <c r="T86" s="3"/>
-      <c r="U86" s="3"/>
-      <c r="V86" s="3"/>
-    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -23968,7 +23784,9 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="3"/>
+      <c r="A80" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="B80" s="3"/>
       <c r="C80" s="3"/>
       <c r="D80" s="3"/>
@@ -23989,6 +23807,7 @@
       <c r="S80" s="3"/>
       <c r="T80" s="3"/>
       <c r="U80" s="3"/>
+      <c r="V80" s="3"/>
     </row>
     <row r="81">
       <c r="A81" s="3"/>
@@ -24159,32 +23978,6 @@
       <c r="U85" s="3"/>
       <c r="V85" s="3"/>
     </row>
-    <row r="86">
-      <c r="A86" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B86" s="3"/>
-      <c r="C86" s="3"/>
-      <c r="D86" s="3"/>
-      <c r="E86" s="3"/>
-      <c r="F86" s="3"/>
-      <c r="G86" s="3"/>
-      <c r="H86" s="3"/>
-      <c r="I86" s="3"/>
-      <c r="J86" s="3"/>
-      <c r="K86" s="3"/>
-      <c r="L86" s="3"/>
-      <c r="M86" s="3"/>
-      <c r="N86" s="3"/>
-      <c r="O86" s="3"/>
-      <c r="P86" s="3"/>
-      <c r="Q86" s="3"/>
-      <c r="R86" s="3"/>
-      <c r="S86" s="3"/>
-      <c r="T86" s="3"/>
-      <c r="U86" s="3"/>
-      <c r="V86" s="3"/>
-    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -26280,7 +26073,9 @@
       <c r="U78" s="3"/>
     </row>
     <row r="79">
-      <c r="A79" s="3"/>
+      <c r="A79" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="B79" s="3"/>
       <c r="C79" s="3"/>
       <c r="D79" s="3"/>
@@ -26301,6 +26096,7 @@
       <c r="S79" s="3"/>
       <c r="T79" s="3"/>
       <c r="U79" s="3"/>
+      <c r="V79" s="3"/>
     </row>
     <row r="80">
       <c r="A80" s="3"/>
@@ -26500,32 +26296,6 @@
       <c r="U85" s="3"/>
       <c r="V85" s="3"/>
     </row>
-    <row r="86">
-      <c r="A86" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B86" s="3"/>
-      <c r="C86" s="3"/>
-      <c r="D86" s="3"/>
-      <c r="E86" s="3"/>
-      <c r="F86" s="3"/>
-      <c r="G86" s="3"/>
-      <c r="H86" s="3"/>
-      <c r="I86" s="3"/>
-      <c r="J86" s="3"/>
-      <c r="K86" s="3"/>
-      <c r="L86" s="3"/>
-      <c r="M86" s="3"/>
-      <c r="N86" s="3"/>
-      <c r="O86" s="3"/>
-      <c r="P86" s="3"/>
-      <c r="Q86" s="3"/>
-      <c r="R86" s="3"/>
-      <c r="S86" s="3"/>
-      <c r="T86" s="3"/>
-      <c r="U86" s="3"/>
-      <c r="V86" s="3"/>
-    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -28702,7 +28472,9 @@
       <c r="U79" s="3"/>
     </row>
     <row r="80">
-      <c r="A80" s="3"/>
+      <c r="A80" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="B80" s="3"/>
       <c r="C80" s="3"/>
       <c r="D80" s="3"/>
@@ -28887,31 +28659,6 @@
       <c r="T85" s="3"/>
       <c r="U85" s="3"/>
     </row>
-    <row r="86">
-      <c r="A86" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B86" s="3"/>
-      <c r="C86" s="3"/>
-      <c r="D86" s="3"/>
-      <c r="E86" s="3"/>
-      <c r="F86" s="3"/>
-      <c r="G86" s="3"/>
-      <c r="H86" s="3"/>
-      <c r="I86" s="3"/>
-      <c r="J86" s="3"/>
-      <c r="K86" s="3"/>
-      <c r="L86" s="3"/>
-      <c r="M86" s="3"/>
-      <c r="N86" s="3"/>
-      <c r="O86" s="3"/>
-      <c r="P86" s="3"/>
-      <c r="Q86" s="3"/>
-      <c r="R86" s="3"/>
-      <c r="S86" s="3"/>
-      <c r="T86" s="3"/>
-      <c r="U86" s="3"/>
-    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -31001,7 +30748,9 @@
       <c r="U78" s="3"/>
     </row>
     <row r="79">
-      <c r="A79" s="3"/>
+      <c r="A79" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="B79" s="3"/>
       <c r="C79" s="3"/>
       <c r="D79" s="3"/>
@@ -31022,6 +30771,7 @@
       <c r="S79" s="3"/>
       <c r="T79" s="3"/>
       <c r="U79" s="3"/>
+      <c r="V79" s="3"/>
     </row>
     <row r="80">
       <c r="A80" s="3"/>
@@ -31243,32 +30993,6 @@
       </c>
       <c r="V85" s="2"/>
     </row>
-    <row r="86">
-      <c r="A86" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B86" s="3"/>
-      <c r="C86" s="3"/>
-      <c r="D86" s="3"/>
-      <c r="E86" s="3"/>
-      <c r="F86" s="3"/>
-      <c r="G86" s="3"/>
-      <c r="H86" s="3"/>
-      <c r="I86" s="3"/>
-      <c r="J86" s="3"/>
-      <c r="K86" s="3"/>
-      <c r="L86" s="3"/>
-      <c r="M86" s="3"/>
-      <c r="N86" s="3"/>
-      <c r="O86" s="3"/>
-      <c r="P86" s="3"/>
-      <c r="Q86" s="3"/>
-      <c r="R86" s="3"/>
-      <c r="S86" s="3"/>
-      <c r="T86" s="3"/>
-      <c r="U86" s="3"/>
-      <c r="V86" s="3"/>
-    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -33420,7 +33144,9 @@
       <c r="U78" s="3"/>
     </row>
     <row r="79">
-      <c r="A79" s="3"/>
+      <c r="A79" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="B79" s="3"/>
       <c r="C79" s="3"/>
       <c r="D79" s="3"/>
@@ -33441,6 +33167,7 @@
       <c r="S79" s="3"/>
       <c r="T79" s="3"/>
       <c r="U79" s="3"/>
+      <c r="V79" s="3"/>
     </row>
     <row r="80">
       <c r="A80" s="3"/>
@@ -33654,32 +33381,6 @@
       <c r="U85" s="2"/>
       <c r="V85" s="2"/>
     </row>
-    <row r="86">
-      <c r="A86" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B86" s="3"/>
-      <c r="C86" s="3"/>
-      <c r="D86" s="3"/>
-      <c r="E86" s="3"/>
-      <c r="F86" s="3"/>
-      <c r="G86" s="3"/>
-      <c r="H86" s="3"/>
-      <c r="I86" s="3"/>
-      <c r="J86" s="3"/>
-      <c r="K86" s="3"/>
-      <c r="L86" s="3"/>
-      <c r="M86" s="3"/>
-      <c r="N86" s="3"/>
-      <c r="O86" s="3"/>
-      <c r="P86" s="3"/>
-      <c r="Q86" s="3"/>
-      <c r="R86" s="3"/>
-      <c r="S86" s="3"/>
-      <c r="T86" s="3"/>
-      <c r="U86" s="3"/>
-      <c r="V86" s="3"/>
-    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -35813,7 +35514,9 @@
       <c r="U78" s="3"/>
     </row>
     <row r="79">
-      <c r="A79" s="3"/>
+      <c r="A79" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="B79" s="3"/>
       <c r="C79" s="3"/>
       <c r="D79" s="3"/>
@@ -35834,6 +35537,7 @@
       <c r="S79" s="3"/>
       <c r="T79" s="3"/>
       <c r="U79" s="3"/>
+      <c r="V79" s="3"/>
     </row>
     <row r="80">
       <c r="A80" s="3"/>
@@ -36047,32 +35751,6 @@
       </c>
       <c r="V85" s="2"/>
     </row>
-    <row r="86">
-      <c r="A86" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B86" s="3"/>
-      <c r="C86" s="3"/>
-      <c r="D86" s="3"/>
-      <c r="E86" s="3"/>
-      <c r="F86" s="3"/>
-      <c r="G86" s="3"/>
-      <c r="H86" s="3"/>
-      <c r="I86" s="3"/>
-      <c r="J86" s="3"/>
-      <c r="K86" s="3"/>
-      <c r="L86" s="3"/>
-      <c r="M86" s="3"/>
-      <c r="N86" s="3"/>
-      <c r="O86" s="3"/>
-      <c r="P86" s="3"/>
-      <c r="Q86" s="3"/>
-      <c r="R86" s="3"/>
-      <c r="S86" s="3"/>
-      <c r="T86" s="3"/>
-      <c r="U86" s="3"/>
-      <c r="V86" s="3"/>
-    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -38181,7 +37859,9 @@
       <c r="U79" s="3"/>
     </row>
     <row r="80">
-      <c r="A80" s="3"/>
+      <c r="A80" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="B80" s="3"/>
       <c r="C80" s="3"/>
       <c r="D80" s="3"/>
@@ -38202,6 +37882,7 @@
       <c r="S80" s="3"/>
       <c r="T80" s="3"/>
       <c r="U80" s="3"/>
+      <c r="V80" s="3"/>
     </row>
     <row r="81">
       <c r="A81" s="3"/>
@@ -38392,32 +38073,6 @@
       <c r="U85" s="3"/>
       <c r="V85" s="3"/>
     </row>
-    <row r="86">
-      <c r="A86" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B86" s="3"/>
-      <c r="C86" s="3"/>
-      <c r="D86" s="3"/>
-      <c r="E86" s="3"/>
-      <c r="F86" s="3"/>
-      <c r="G86" s="3"/>
-      <c r="H86" s="3"/>
-      <c r="I86" s="3"/>
-      <c r="J86" s="3"/>
-      <c r="K86" s="3"/>
-      <c r="L86" s="3"/>
-      <c r="M86" s="3"/>
-      <c r="N86" s="3"/>
-      <c r="O86" s="3"/>
-      <c r="P86" s="3"/>
-      <c r="Q86" s="3"/>
-      <c r="R86" s="3"/>
-      <c r="S86" s="3"/>
-      <c r="T86" s="3"/>
-      <c r="U86" s="3"/>
-      <c r="V86" s="3"/>
-    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -40511,7 +40166,9 @@
       <c r="U78" s="3"/>
     </row>
     <row r="79">
-      <c r="A79" s="3"/>
+      <c r="A79" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="B79" s="3"/>
       <c r="C79" s="3"/>
       <c r="D79" s="3"/>
@@ -40532,6 +40189,7 @@
       <c r="S79" s="3"/>
       <c r="T79" s="3"/>
       <c r="U79" s="3"/>
+      <c r="V79" s="3"/>
     </row>
     <row r="80">
       <c r="A80" s="3"/>
@@ -40727,32 +40385,6 @@
       <c r="U85" s="3"/>
       <c r="V85" s="3"/>
     </row>
-    <row r="86">
-      <c r="A86" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B86" s="3"/>
-      <c r="C86" s="3"/>
-      <c r="D86" s="3"/>
-      <c r="E86" s="3"/>
-      <c r="F86" s="3"/>
-      <c r="G86" s="3"/>
-      <c r="H86" s="3"/>
-      <c r="I86" s="3"/>
-      <c r="J86" s="3"/>
-      <c r="K86" s="3"/>
-      <c r="L86" s="3"/>
-      <c r="M86" s="3"/>
-      <c r="N86" s="3"/>
-      <c r="O86" s="3"/>
-      <c r="P86" s="3"/>
-      <c r="Q86" s="3"/>
-      <c r="R86" s="3"/>
-      <c r="S86" s="3"/>
-      <c r="T86" s="3"/>
-      <c r="U86" s="3"/>
-      <c r="V86" s="3"/>
-    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -42912,7 +42544,9 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="3"/>
+      <c r="A81" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="B81" s="3"/>
       <c r="C81" s="3"/>
       <c r="D81" s="3"/>
@@ -42933,6 +42567,7 @@
       <c r="S81" s="3"/>
       <c r="T81" s="3"/>
       <c r="U81" s="3"/>
+      <c r="V81" s="3"/>
     </row>
     <row r="82">
       <c r="A82" s="1" t="s">
@@ -43077,32 +42712,6 @@
       <c r="T85" s="3"/>
       <c r="U85" s="3"/>
       <c r="V85" s="3"/>
-    </row>
-    <row r="86">
-      <c r="A86" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B86" s="3"/>
-      <c r="C86" s="3"/>
-      <c r="D86" s="3"/>
-      <c r="E86" s="3"/>
-      <c r="F86" s="3"/>
-      <c r="G86" s="3"/>
-      <c r="H86" s="3"/>
-      <c r="I86" s="3"/>
-      <c r="J86" s="3"/>
-      <c r="K86" s="3"/>
-      <c r="L86" s="3"/>
-      <c r="M86" s="3"/>
-      <c r="N86" s="3"/>
-      <c r="O86" s="3"/>
-      <c r="P86" s="3"/>
-      <c r="Q86" s="3"/>
-      <c r="R86" s="3"/>
-      <c r="S86" s="3"/>
-      <c r="T86" s="3"/>
-      <c r="U86" s="3"/>
-      <c r="V86" s="3"/>
     </row>
   </sheetData>
   <drawing r:id="rId1"/>
@@ -54993,7 +54602,9 @@
       <c r="U79" s="3"/>
     </row>
     <row r="80">
-      <c r="A80" s="3"/>
+      <c r="A80" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="B80" s="3"/>
       <c r="C80" s="3"/>
       <c r="D80" s="3"/>
@@ -55178,31 +54789,6 @@
       <c r="T85" s="3"/>
       <c r="U85" s="3"/>
     </row>
-    <row r="86">
-      <c r="A86" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B86" s="3"/>
-      <c r="C86" s="3"/>
-      <c r="D86" s="3"/>
-      <c r="E86" s="3"/>
-      <c r="F86" s="3"/>
-      <c r="G86" s="3"/>
-      <c r="H86" s="3"/>
-      <c r="I86" s="3"/>
-      <c r="J86" s="3"/>
-      <c r="K86" s="3"/>
-      <c r="L86" s="3"/>
-      <c r="M86" s="3"/>
-      <c r="N86" s="3"/>
-      <c r="O86" s="3"/>
-      <c r="P86" s="3"/>
-      <c r="Q86" s="3"/>
-      <c r="R86" s="3"/>
-      <c r="S86" s="3"/>
-      <c r="T86" s="3"/>
-      <c r="U86" s="3"/>
-    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -62136,7 +61722,9 @@
       <c r="U78" s="3"/>
     </row>
     <row r="79">
-      <c r="A79" s="3"/>
+      <c r="A79" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="B79" s="3"/>
       <c r="C79" s="3"/>
       <c r="D79" s="3"/>
@@ -62344,31 +61932,6 @@
       <c r="T85" s="3"/>
       <c r="U85" s="3"/>
     </row>
-    <row r="86">
-      <c r="A86" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B86" s="3"/>
-      <c r="C86" s="3"/>
-      <c r="D86" s="3"/>
-      <c r="E86" s="3"/>
-      <c r="F86" s="3"/>
-      <c r="G86" s="3"/>
-      <c r="H86" s="3"/>
-      <c r="I86" s="3"/>
-      <c r="J86" s="3"/>
-      <c r="K86" s="3"/>
-      <c r="L86" s="3"/>
-      <c r="M86" s="3"/>
-      <c r="N86" s="3"/>
-      <c r="O86" s="3"/>
-      <c r="P86" s="3"/>
-      <c r="Q86" s="3"/>
-      <c r="R86" s="3"/>
-      <c r="S86" s="3"/>
-      <c r="T86" s="3"/>
-      <c r="U86" s="3"/>
-    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -64713,7 +64276,9 @@
       <c r="W77" s="3"/>
     </row>
     <row r="78">
-      <c r="A78" s="3"/>
+      <c r="A78" s="2" t="s">
+        <v>16</v>
+      </c>
       <c r="B78" s="3"/>
       <c r="C78" s="3"/>
       <c r="D78" s="3"/>
@@ -64731,10 +64296,14 @@
       <c r="P78" s="3"/>
       <c r="Q78" s="3"/>
       <c r="R78" s="3"/>
-      <c r="S78" s="3"/>
-      <c r="T78" s="3"/>
-      <c r="U78" s="3"/>
-      <c r="V78" s="3"/>
+      <c r="S78" s="2">
+        <v>20.0</v>
+      </c>
+      <c r="T78" s="2"/>
+      <c r="U78" s="2">
+        <v>1.0</v>
+      </c>
+      <c r="V78" s="2"/>
       <c r="W78" s="3"/>
     </row>
     <row r="79">
@@ -64923,37 +64492,6 @@
       <c r="V84" s="3"/>
       <c r="W84" s="3"/>
     </row>
-    <row r="85">
-      <c r="A85" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B85" s="3"/>
-      <c r="C85" s="3"/>
-      <c r="D85" s="3"/>
-      <c r="E85" s="3"/>
-      <c r="F85" s="3"/>
-      <c r="G85" s="3"/>
-      <c r="H85" s="3"/>
-      <c r="I85" s="3"/>
-      <c r="J85" s="3"/>
-      <c r="K85" s="3"/>
-      <c r="L85" s="3"/>
-      <c r="M85" s="3"/>
-      <c r="N85" s="3"/>
-      <c r="O85" s="3"/>
-      <c r="P85" s="3"/>
-      <c r="Q85" s="3"/>
-      <c r="R85" s="3"/>
-      <c r="S85" s="2">
-        <v>20.0</v>
-      </c>
-      <c r="T85" s="2"/>
-      <c r="U85" s="2">
-        <v>1.0</v>
-      </c>
-      <c r="V85" s="2"/>
-      <c r="W85" s="3"/>
-    </row>
     <row r="86">
       <c r="A86" s="3"/>
       <c r="B86" s="3"/>
@@ -67799,12 +67337,16 @@
       <c r="W78" s="3"/>
     </row>
     <row r="79">
-      <c r="A79" s="3"/>
+      <c r="A79" s="2" t="s">
+        <v>16</v>
+      </c>
       <c r="B79" s="3"/>
       <c r="C79" s="3"/>
       <c r="D79" s="3"/>
-      <c r="E79" s="3"/>
-      <c r="F79" s="3"/>
+      <c r="E79" s="2">
+        <v>2.0</v>
+      </c>
+      <c r="F79" s="2"/>
       <c r="G79" s="3"/>
       <c r="H79" s="3"/>
       <c r="I79" s="3"/>
@@ -67817,8 +67359,10 @@
       <c r="P79" s="3"/>
       <c r="Q79" s="3"/>
       <c r="R79" s="3"/>
-      <c r="S79" s="3"/>
-      <c r="T79" s="3"/>
+      <c r="S79" s="2">
+        <v>1.0</v>
+      </c>
+      <c r="T79" s="2"/>
       <c r="U79" s="3"/>
       <c r="V79" s="3"/>
       <c r="W79" s="3"/>
@@ -68003,37 +67547,6 @@
       <c r="V85" s="3"/>
       <c r="W85" s="3"/>
     </row>
-    <row r="86">
-      <c r="A86" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B86" s="3"/>
-      <c r="C86" s="3"/>
-      <c r="D86" s="3"/>
-      <c r="E86" s="2">
-        <v>2.0</v>
-      </c>
-      <c r="F86" s="2"/>
-      <c r="G86" s="3"/>
-      <c r="H86" s="3"/>
-      <c r="I86" s="3"/>
-      <c r="J86" s="3"/>
-      <c r="K86" s="3"/>
-      <c r="L86" s="3"/>
-      <c r="M86" s="3"/>
-      <c r="N86" s="3"/>
-      <c r="O86" s="3"/>
-      <c r="P86" s="3"/>
-      <c r="Q86" s="3"/>
-      <c r="R86" s="3"/>
-      <c r="S86" s="2">
-        <v>1.0</v>
-      </c>
-      <c r="T86" s="2"/>
-      <c r="U86" s="3"/>
-      <c r="V86" s="3"/>
-      <c r="W86" s="3"/>
-    </row>
     <row r="87">
       <c r="A87" s="3"/>
       <c r="B87" s="3"/>
@@ -70886,10 +70399,14 @@
       <c r="W79" s="3"/>
     </row>
     <row r="80">
-      <c r="A80" s="3"/>
-      <c r="B80" s="3"/>
-      <c r="C80" s="3"/>
-      <c r="D80" s="3"/>
+      <c r="A80" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B80" s="2"/>
+      <c r="C80" s="2">
+        <v>13.0</v>
+      </c>
+      <c r="D80" s="2"/>
       <c r="E80" s="3"/>
       <c r="F80" s="3"/>
       <c r="G80" s="3"/>
@@ -71069,35 +70586,6 @@
       <c r="V85" s="3"/>
       <c r="W85" s="3"/>
     </row>
-    <row r="86">
-      <c r="A86" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B86" s="2"/>
-      <c r="C86" s="2">
-        <v>13.0</v>
-      </c>
-      <c r="D86" s="2"/>
-      <c r="E86" s="3"/>
-      <c r="F86" s="3"/>
-      <c r="G86" s="3"/>
-      <c r="H86" s="3"/>
-      <c r="I86" s="3"/>
-      <c r="J86" s="3"/>
-      <c r="K86" s="3"/>
-      <c r="L86" s="3"/>
-      <c r="M86" s="3"/>
-      <c r="N86" s="3"/>
-      <c r="O86" s="3"/>
-      <c r="P86" s="3"/>
-      <c r="Q86" s="3"/>
-      <c r="R86" s="3"/>
-      <c r="S86" s="3"/>
-      <c r="T86" s="3"/>
-      <c r="U86" s="3"/>
-      <c r="V86" s="3"/>
-      <c r="W86" s="3"/>
-    </row>
     <row r="87">
       <c r="A87" s="3"/>
       <c r="B87" s="3"/>
@@ -73722,27 +73210,42 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="3"/>
+      <c r="A80" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="B80" s="3"/>
       <c r="C80" s="3"/>
       <c r="D80" s="3"/>
       <c r="E80" s="3"/>
       <c r="F80" s="3"/>
-      <c r="G80" s="3"/>
-      <c r="H80" s="3"/>
-      <c r="I80" s="3"/>
-      <c r="J80" s="3"/>
-      <c r="K80" s="3"/>
-      <c r="L80" s="3"/>
-      <c r="M80" s="3"/>
-      <c r="N80" s="3"/>
-      <c r="O80" s="3"/>
-      <c r="P80" s="3"/>
+      <c r="G80" s="2">
+        <v>15.0</v>
+      </c>
+      <c r="H80" s="2"/>
+      <c r="I80" s="2">
+        <v>1.0</v>
+      </c>
+      <c r="J80" s="2"/>
+      <c r="K80" s="2">
+        <v>10.0</v>
+      </c>
+      <c r="L80" s="2"/>
+      <c r="M80" s="2">
+        <v>5.0</v>
+      </c>
+      <c r="N80" s="2"/>
+      <c r="O80" s="2">
+        <v>10.0</v>
+      </c>
+      <c r="P80" s="2"/>
       <c r="Q80" s="3"/>
       <c r="R80" s="3"/>
       <c r="S80" s="3"/>
       <c r="T80" s="3"/>
-      <c r="U80" s="3"/>
+      <c r="U80" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="V80" s="2"/>
     </row>
     <row r="81">
       <c r="A81" s="3"/>
@@ -73923,44 +73426,6 @@
       <c r="U85" s="3"/>
       <c r="V85" s="3"/>
     </row>
-    <row r="86">
-      <c r="A86" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B86" s="3"/>
-      <c r="C86" s="3"/>
-      <c r="D86" s="3"/>
-      <c r="E86" s="3"/>
-      <c r="F86" s="3"/>
-      <c r="G86" s="2">
-        <v>15.0</v>
-      </c>
-      <c r="H86" s="2"/>
-      <c r="I86" s="2">
-        <v>1.0</v>
-      </c>
-      <c r="J86" s="2"/>
-      <c r="K86" s="2">
-        <v>10.0</v>
-      </c>
-      <c r="L86" s="2"/>
-      <c r="M86" s="2">
-        <v>5.0</v>
-      </c>
-      <c r="N86" s="2"/>
-      <c r="O86" s="2">
-        <v>10.0</v>
-      </c>
-      <c r="P86" s="2"/>
-      <c r="Q86" s="3"/>
-      <c r="R86" s="3"/>
-      <c r="S86" s="3"/>
-      <c r="T86" s="3"/>
-      <c r="U86" s="2">
-        <v>30.0</v>
-      </c>
-      <c r="V86" s="2"/>
-    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -76106,14 +75571,18 @@
       <c r="U78" s="3"/>
     </row>
     <row r="79">
-      <c r="A79" s="3"/>
+      <c r="A79" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="B79" s="3"/>
       <c r="C79" s="3"/>
       <c r="D79" s="3"/>
       <c r="E79" s="3"/>
       <c r="F79" s="3"/>
-      <c r="G79" s="3"/>
-      <c r="H79" s="3"/>
+      <c r="G79" s="2">
+        <v>1.0</v>
+      </c>
+      <c r="H79" s="2"/>
       <c r="I79" s="3"/>
       <c r="J79" s="3"/>
       <c r="K79" s="3"/>
@@ -76127,6 +75596,7 @@
       <c r="S79" s="3"/>
       <c r="T79" s="3"/>
       <c r="U79" s="3"/>
+      <c r="V79" s="3"/>
     </row>
     <row r="80">
       <c r="A80" s="3"/>
@@ -76320,34 +75790,6 @@
       <c r="U85" s="3"/>
       <c r="V85" s="3"/>
     </row>
-    <row r="86">
-      <c r="A86" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B86" s="3"/>
-      <c r="C86" s="3"/>
-      <c r="D86" s="3"/>
-      <c r="E86" s="3"/>
-      <c r="F86" s="3"/>
-      <c r="G86" s="2">
-        <v>1.0</v>
-      </c>
-      <c r="H86" s="2"/>
-      <c r="I86" s="3"/>
-      <c r="J86" s="3"/>
-      <c r="K86" s="3"/>
-      <c r="L86" s="3"/>
-      <c r="M86" s="3"/>
-      <c r="N86" s="3"/>
-      <c r="O86" s="3"/>
-      <c r="P86" s="3"/>
-      <c r="Q86" s="3"/>
-      <c r="R86" s="3"/>
-      <c r="S86" s="3"/>
-      <c r="T86" s="3"/>
-      <c r="U86" s="3"/>
-      <c r="V86" s="3"/>
-    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>